<commit_message>
22-04-2026 /Unit based hirearchy development in process
</commit_message>
<xml_diff>
--- a/test_default.xlsx
+++ b/test_default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\AmazonDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527C66CF-60D9-4165-B687-928766AD0333}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC85D26-C24A-4C81-8FDC-064482DC001A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fixed Assets" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
   <si>
     <t>Yes</t>
   </si>
@@ -254,10 +254,13 @@
     <t>Testing of process owner on excel file upload. Also reminder frequency</t>
   </si>
   <si>
-    <t>Weekly</t>
-  </si>
-  <si>
     <t>a</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>divyeshparmar0548@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -428,7 +431,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
@@ -574,6 +577,9 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="11" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -1257,7 +1263,7 @@
       </c>
       <c r="G7" s="43"/>
       <c r="H7" s="45" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
@@ -1296,13 +1302,13 @@
         <v>42</v>
       </c>
       <c r="W7" s="17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="X7" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="Y7" s="17" t="s">
-        <v>48</v>
+      <c r="Y7" s="49" t="s">
+        <v>61</v>
       </c>
       <c r="Z7" s="17" t="s">
         <v>3</v>
@@ -1959,8 +1965,11 @@
       <formula1>"P, O"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="Y7" r:id="rId1" xr:uid="{26F91A05-2719-4714-AEB5-D52B67565B9E}"/>
+  </hyperlinks>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup scale="22" orientation="landscape" r:id="rId1"/>
+  <pageSetup scale="22" orientation="landscape" r:id="rId2"/>
   <headerFooter alignWithMargins="0">
     <oddHeader>&amp;C&amp;"-,Bold"Gujarat Fluorochemicals Limited</oddHeader>
     <oddFooter>&amp;C&amp;"-,Italic"&amp;9&amp;K00-033Private and Confidential&amp;R&amp;"Calibri,Regular"&amp;9&amp;P</oddFooter>

</xml_diff>

<commit_message>
Unit based IFC flow
</commit_message>
<xml_diff>
--- a/test_default.xlsx
+++ b/test_default.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Divyesh\IFC\AmazonDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FC85D26-C24A-4C81-8FDC-064482DC001A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B630DE1A-0AC0-461B-BDAC-F201194E3274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Fixed Assets" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="64">
   <si>
     <t>Yes</t>
   </si>
@@ -257,10 +257,16 @@
     <t>a</t>
   </si>
   <si>
-    <t>Daily</t>
-  </si>
-  <si>
-    <t>divyeshparmar0548@gmail.com</t>
+    <t>user3xyz@gmail.com</t>
+  </si>
+  <si>
+    <t>Quarterly</t>
+  </si>
+  <si>
+    <t>FA02</t>
+  </si>
+  <si>
+    <t>user2xyz@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -568,6 +574,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="11" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -577,9 +586,6 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="11" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="12">
@@ -967,11 +973,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="48" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
       <c r="D1" s="26" t="s">
         <v>53</v>
       </c>
@@ -1003,11 +1009,11 @@
       <c r="AD1" s="2"/>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
       <c r="D2" s="27" t="s">
         <v>49</v>
       </c>
@@ -1043,11 +1049,11 @@
       <c r="AD2" s="2"/>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A3" s="47" t="s">
+      <c r="A3" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="B3" s="47"/>
-      <c r="C3" s="47"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
       <c r="D3" s="12" t="s">
         <v>36</v>
       </c>
@@ -1115,42 +1121,42 @@
       <c r="AD4" s="2"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="A5" s="48" t="s">
+      <c r="A5" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
+      <c r="B5" s="49"/>
+      <c r="C5" s="49"/>
+      <c r="D5" s="49"/>
+      <c r="E5" s="49"/>
       <c r="F5" s="37"/>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="48"/>
-      <c r="I5" s="48"/>
-      <c r="J5" s="48"/>
-      <c r="K5" s="48"/>
-      <c r="L5" s="46" t="s">
+      <c r="H5" s="49"/>
+      <c r="I5" s="49"/>
+      <c r="J5" s="49"/>
+      <c r="K5" s="49"/>
+      <c r="L5" s="47" t="s">
         <v>33</v>
       </c>
-      <c r="M5" s="46"/>
-      <c r="N5" s="46"/>
-      <c r="O5" s="46"/>
-      <c r="P5" s="46"/>
-      <c r="Q5" s="46"/>
-      <c r="R5" s="46"/>
-      <c r="S5" s="46"/>
-      <c r="T5" s="46"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="46"/>
-      <c r="W5" s="46"/>
-      <c r="X5" s="46"/>
-      <c r="Y5" s="46"/>
-      <c r="Z5" s="46"/>
-      <c r="AA5" s="46"/>
-      <c r="AB5" s="46"/>
-      <c r="AC5" s="46"/>
-      <c r="AD5" s="46"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="47"/>
+      <c r="O5" s="47"/>
+      <c r="P5" s="47"/>
+      <c r="Q5" s="47"/>
+      <c r="R5" s="47"/>
+      <c r="S5" s="47"/>
+      <c r="T5" s="47"/>
+      <c r="U5" s="47"/>
+      <c r="V5" s="47"/>
+      <c r="W5" s="47"/>
+      <c r="X5" s="47"/>
+      <c r="Y5" s="47"/>
+      <c r="Z5" s="47"/>
+      <c r="AA5" s="47"/>
+      <c r="AB5" s="47"/>
+      <c r="AC5" s="47"/>
+      <c r="AD5" s="47"/>
     </row>
     <row r="6" spans="1:31" s="5" customFormat="1" ht="120.75" x14ac:dyDescent="0.2">
       <c r="A6" s="28" t="s">
@@ -1302,13 +1308,13 @@
         <v>42</v>
       </c>
       <c r="W7" s="17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="X7" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="Y7" s="49" t="s">
-        <v>61</v>
+      <c r="Y7" s="46" t="s">
+        <v>60</v>
       </c>
       <c r="Z7" s="17" t="s">
         <v>3</v>
@@ -1325,37 +1331,92 @@
       <c r="AD7" s="42"/>
       <c r="AE7" s="44"/>
     </row>
-    <row r="8" spans="1:31" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="20"/>
-      <c r="M8" s="19"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="16"/>
-      <c r="S8" s="17"/>
-      <c r="T8" s="17"/>
-      <c r="U8" s="17"/>
-      <c r="V8" s="17"/>
-      <c r="W8" s="17"/>
-      <c r="X8" s="21"/>
-      <c r="Y8" s="21"/>
-      <c r="Z8" s="17"/>
-      <c r="AA8" s="19"/>
-      <c r="AB8" s="18"/>
-      <c r="AC8" s="21"/>
-      <c r="AD8" s="21"/>
+    <row r="8" spans="1:31" ht="102" x14ac:dyDescent="0.2">
+      <c r="A8" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="30" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="43"/>
+      <c r="H8" s="45" t="s">
+        <v>59</v>
+      </c>
+      <c r="I8" s="43"/>
+      <c r="J8" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="K8" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="L8" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="M8" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="N8" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="O8" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="P8" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="R8" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="S8" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="T8" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="U8" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="V8" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="W8" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="X8" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y8" s="46" t="s">
+        <v>63</v>
+      </c>
+      <c r="Z8" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA8" s="35" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="AC8" s="36" t="s">
+        <v>44</v>
+      </c>
+      <c r="AD8" s="42"/>
+      <c r="AE8" s="44"/>
     </row>
     <row r="9" spans="1:31" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="10"/>
@@ -1957,19 +2018,20 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="S7:S25" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Preventive,Detective"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB15:AB19 AB8 AB23 AB10:AB13" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AB15:AB19 AB10:AB13 AB23" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Effective, Ineffective - Design Gap, Ineffective - Implementation Gap"</formula1>
     </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="X7:X25 Y7:Y1048576" xr:uid="{00000000-0002-0000-0000-000005000000}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Y7:Y1048576 X7:X25" xr:uid="{00000000-0002-0000-0000-000005000000}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G27 I27 K27:K30" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"P, O"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="Y7" r:id="rId1" xr:uid="{26F91A05-2719-4714-AEB5-D52B67565B9E}"/>
+    <hyperlink ref="Y8" r:id="rId2" xr:uid="{EE13AA4E-81B0-45EB-A349-CFFB82685891}"/>
   </hyperlinks>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup scale="22" orientation="landscape" r:id="rId2"/>
+  <pageSetup scale="22" orientation="landscape" r:id="rId3"/>
   <headerFooter alignWithMargins="0">
     <oddHeader>&amp;C&amp;"-,Bold"Gujarat Fluorochemicals Limited</oddHeader>
     <oddFooter>&amp;C&amp;"-,Italic"&amp;9&amp;K00-033Private and Confidential&amp;R&amp;"Calibri,Regular"&amp;9&amp;P</oddFooter>

</xml_diff>